<commit_message>
Implement standalone mode for Gitai Earthmovers app, allowing local usage of Gitai.xlsx without internet. Update connection and save status badges in the UI. Enhance API client for session management and data persistence. Add scripts for applying payment data and receipts to the Excel file. Include detailed documentation for standalone app usage and workflow.
</commit_message>
<xml_diff>
--- a/Gitai.xlsx
+++ b/Gitai.xlsx
@@ -24085,7 +24085,7 @@
         <v>48399</v>
       </c>
       <c r="E26" t="str">
-        <v>2024-01-28</v>
+        <v>2024-01-29</v>
       </c>
       <c r="F26" t="str">
         <v>0</v>
@@ -24100,7 +24100,7 @@
         <v>Paid</v>
       </c>
       <c r="J26" t="str">
-        <v>P:34455 I:13944</v>
+        <v>P:34455 I:13944 | TXN7388832616 GB0129989356 Completed 29-01-2024</v>
       </c>
     </row>
     <row r="27">
@@ -24132,7 +24132,7 @@
         <v>Paid</v>
       </c>
       <c r="J27" t="str">
-        <v>P:34773 I:13626</v>
+        <v>P:34773 I:13626 | TXN5863354926 Failed then TXN5906895034 GB0228746203 Completed 28-02-2024</v>
       </c>
     </row>
     <row r="28">
@@ -24187,16 +24187,16 @@
         <v>0</v>
       </c>
       <c r="G29" t="str">
-        <v>0</v>
+        <v>1620</v>
       </c>
       <c r="H29" t="str">
-        <v>48399</v>
+        <v>50019</v>
       </c>
       <c r="I29" t="str">
         <v>Paid</v>
       </c>
       <c r="J29" t="str">
-        <v>P:35418 I:12981</v>
+        <v>P:35418 I:12981 | TXN4828640519 GB0504159679 penalty ₹1,620 Completed 04-05-2024</v>
       </c>
     </row>
     <row r="30">
@@ -24277,22 +24277,22 @@
         <v>48399</v>
       </c>
       <c r="E32" t="str">
-        <v>2024-07-28</v>
+        <v>2024-07-31</v>
       </c>
       <c r="F32" t="str">
-        <v>0</v>
+        <v>895</v>
       </c>
       <c r="G32" t="str">
         <v>0</v>
       </c>
       <c r="H32" t="str">
-        <v>48399</v>
+        <v>49294</v>
       </c>
       <c r="I32" t="str">
         <v>Paid</v>
       </c>
       <c r="J32" t="str">
-        <v>P:36408 I:11991</v>
+        <v>P:36408 I:11991 | TXN3578603114 GB0731619886 Completed 31-07-2024; TXN4289021146 fee ₹119 02-08-2024</v>
       </c>
     </row>
     <row r="33">
@@ -24341,22 +24341,22 @@
         <v>48399</v>
       </c>
       <c r="E34" t="str">
-        <v>2024-09-28</v>
+        <v>2024-10-11</v>
       </c>
       <c r="F34" t="str">
-        <v>0</v>
+        <v>1552</v>
       </c>
       <c r="G34" t="str">
         <v>0</v>
       </c>
       <c r="H34" t="str">
-        <v>48399</v>
+        <v>49951</v>
       </c>
       <c r="I34" t="str">
         <v>Paid</v>
       </c>
       <c r="J34" t="str">
-        <v>P:37083 I:11316</v>
+        <v>P:37083 I:11316 | TXN8333159583 GB1011464183 Completed 11-10-2024 (13 days late)</v>
       </c>
     </row>
     <row r="35">
@@ -24373,22 +24373,22 @@
         <v>48399</v>
       </c>
       <c r="E35" t="str">
-        <v>2024-10-28</v>
+        <v>2024-10-29</v>
       </c>
       <c r="F35" t="str">
-        <v>0</v>
+        <v>736</v>
       </c>
       <c r="G35" t="str">
         <v>0</v>
       </c>
       <c r="H35" t="str">
-        <v>48399</v>
+        <v>49135</v>
       </c>
       <c r="I35" t="str">
         <v>Paid</v>
       </c>
       <c r="J35" t="str">
-        <v>P:37426 I:10973</v>
+        <v>P:37426 I:10973 | TXN8787846197+8829566659 Failed then TXN8973323525 GB1029353789 Completed 29-10-2024</v>
       </c>
     </row>
     <row r="36">
@@ -24437,22 +24437,22 @@
         <v>48399</v>
       </c>
       <c r="E37" t="str">
-        <v>2024-12-28</v>
+        <v>2025-01-07</v>
       </c>
       <c r="F37" t="str">
-        <v>0</v>
+        <v>2068</v>
       </c>
       <c r="G37" t="str">
         <v>0</v>
       </c>
       <c r="H37" t="str">
-        <v>48399</v>
+        <v>50467</v>
       </c>
       <c r="I37" t="str">
         <v>Paid</v>
       </c>
       <c r="J37" t="str">
-        <v>P:38120 I:10279</v>
+        <v>P:38120 I:10279 | TXN7560144060 Failed then TXN7703512396 GB0107818951 Completed 07-01-2025 (inst due 28-12-2024)</v>
       </c>
     </row>
     <row r="38">
@@ -24472,19 +24472,19 @@
         <v>2025-01-28</v>
       </c>
       <c r="F38" t="str">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="G38" t="str">
         <v>0</v>
       </c>
       <c r="H38" t="str">
-        <v>48399</v>
+        <v>48899</v>
       </c>
       <c r="I38" t="str">
         <v>Paid</v>
       </c>
       <c r="J38" t="str">
-        <v>P:38472 I:9927</v>
+        <v>P:38472 I:9927 | TXN5292297051 Failed then TXN5541168306 GB0128660234 Completed 28-01-2025</v>
       </c>
     </row>
     <row r="39">
@@ -24757,22 +24757,22 @@
         <v>48399</v>
       </c>
       <c r="E47" t="str">
-        <v>2025-10-28</v>
+        <v>2025-10-31</v>
       </c>
       <c r="F47" t="str">
-        <v>0</v>
+        <v>3660</v>
       </c>
       <c r="G47" t="str">
         <v>0</v>
       </c>
       <c r="H47" t="str">
-        <v>48399</v>
+        <v>52059</v>
       </c>
       <c r="I47" t="str">
         <v>Paid</v>
       </c>
       <c r="J47" t="str">
-        <v>P:41789 I:6610</v>
+        <v>P:41789 I:6610 | TXN6783731773 GB1031780222 Completed 31-10-2025 (3 days late)</v>
       </c>
     </row>
     <row r="48">
@@ -24836,7 +24836,7 @@
         <v>Paid</v>
       </c>
       <c r="J49" t="str">
-        <v>P:42564 I:5835</v>
+        <v>P:42564 I:5835 | Z97477458/48-1 ACH CLEAR 28-12-2025</v>
       </c>
     </row>
     <row r="50">
@@ -24868,7 +24868,7 @@
         <v>Paid</v>
       </c>
       <c r="J50" t="str">
-        <v>P:42957 I:5442</v>
+        <v>P:42957 I:5442 | Z97477458/49-1 ACH CLEAR 28-01-2026</v>
       </c>
     </row>
     <row r="51">
@@ -24900,7 +24900,7 @@
         <v>Paid</v>
       </c>
       <c r="J51" t="str">
-        <v>P:43354 I:5045</v>
+        <v>P:43354 I:5045 | Z97477458/50-1 ACH CLEAR 28-02-2026</v>
       </c>
     </row>
     <row r="52">
@@ -24917,22 +24917,22 @@
         <v>48399</v>
       </c>
       <c r="E52" t="str">
-        <v>2026-03-28</v>
+        <v>2026-04-08</v>
       </c>
       <c r="F52" t="str">
         <v>0</v>
       </c>
       <c r="G52" t="str">
-        <v>0</v>
+        <v>2029</v>
       </c>
       <c r="H52" t="str">
-        <v>48399</v>
+        <v>50428</v>
       </c>
       <c r="I52" t="str">
         <v>Paid</v>
       </c>
       <c r="J52" t="str">
-        <v>P:43754 I:4645</v>
+        <v>P:43754 I:4645 | Z97477458/51-1 ACH BOUNCE 28-03; RZ97477458/51-1 CHEQUE BOUNCE 04-04; ON357904706+707 CLEAR 08-04; ON357904710 penalty ₹2,029 10-04</v>
       </c>
     </row>
     <row r="53">
@@ -24949,22 +24949,22 @@
         <v>48399</v>
       </c>
       <c r="E53" t="str">
-        <v>2026-04-28</v>
+        <v>2026-05-01</v>
       </c>
       <c r="F53" t="str">
-        <v>0</v>
+        <v>736</v>
       </c>
       <c r="G53" t="str">
         <v>0</v>
       </c>
       <c r="H53" t="str">
-        <v>48399</v>
+        <v>49135</v>
       </c>
       <c r="I53" t="str">
         <v>Paid</v>
       </c>
       <c r="J53" t="str">
-        <v>P:44158 I:4241</v>
+        <v>P:44158 I:4241 | Z97477458/52-1 ACH BOUNCE 28-04; TXN0202348420 GB0501140671 Completed 01-05-2026</v>
       </c>
     </row>
     <row r="54">
@@ -24981,22 +24981,22 @@
         <v>48399</v>
       </c>
       <c r="E54" t="str">
-        <v>2026-05-28</v>
+        <v>2026-06-01</v>
       </c>
       <c r="F54" t="str">
-        <v>0</v>
+        <v>816</v>
       </c>
       <c r="G54" t="str">
         <v>0</v>
       </c>
       <c r="H54" t="str">
-        <v>48399</v>
+        <v>49215</v>
       </c>
       <c r="I54" t="str">
         <v>Paid</v>
       </c>
       <c r="J54" t="str">
-        <v>P:44566 I:3833</v>
+        <v>P:44566 I:3833 | Z97477458/53-1 ACH BOUNCE 28-05; TXN5744964581 GB0601768889 Completed 01-06-2026 2:50 PM</v>
       </c>
     </row>
     <row r="55">
@@ -25405,7 +25405,7 @@
         <v>Monthly</v>
       </c>
       <c r="W2" t="str">
-        <v>Asset cost ₹31,29,698 | Chola repayment schedule 13/06/2026 | Instl 18 partial ₹683.81</v>
+        <v>Chola payments synced 13/06/2026 | 53 EMIs paid | bounce/penalty logged ₹14,612 | Inst 54 due 28-06-2026</v>
       </c>
     </row>
     <row r="3">

</xml_diff>